<commit_message>
feat: novos campus inf estudantes
</commit_message>
<xml_diff>
--- a/template_estudantes.xlsx
+++ b/template_estudantes.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,7 +35,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="007F8C8D"/>
+      <color rgb="005D6D7E"/>
       <sz val="9"/>
     </font>
     <font>
@@ -62,6 +62,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="002C3E50"/>
       <sz val="11"/>
     </font>
@@ -70,8 +76,40 @@
       <color rgb="00C0392B"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A5276"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002C3E50"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00117A65"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006E2F8E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007D6608"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -85,17 +123,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007F8C8D"/>
+        <fgColor rgb="001A5276"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F9EBEA"/>
+        <fgColor rgb="00117A65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDFEFE"/>
+        <fgColor rgb="006E2F8E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007D6608"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -130,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -138,13 +186,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -160,6 +214,27 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -527,29 +602,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="38" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="42" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -558,301 +638,376 @@
           <t>rm_estudante</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ra_estudante</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>nu_chamada</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>nome_estudante</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>serie</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>turma</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>turno</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>data_nascimento</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>email_estudante</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>rg_estudante</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>uf_rg</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>org_emissor_rg</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>cpf_estudante</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>data_ingresso</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>mae_nome</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>mae_telefone</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>mae_email</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>pai_nome</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>pai_telefone</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>pai_email</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>endereco_estudante</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="W1" s="5" t="inlineStr">
         <is>
           <t>termo_autorizado</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>foto_coletada</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="Y1" s="5" t="inlineStr">
         <is>
           <t>observacoes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Matrícula/RM do estudante (ex: 006810)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Matrícula/RM do estudante (ex: 006810)  ★ OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Registro do Aluno SESI (ex: 000120628062-1)</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Nome completo (ex: ANA BEATRIZ SILVA SANTOS)</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Série (ex: 6º Ano | 7º Ano | 8º Ano | 9º Ano | 1º EM | 2º EM | 3º EM)</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Turma (ex: A | B | C)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Turno (ex: Manhã | Tarde | Integral)</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Número de chamada na turma (ex: 01)</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Nome completo do estudante (ex: ANA BEATRIZ SILVA SANTOS)  ★ OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Série: 6º Ano | 7º Ano | 8º Ano | 9º Ano | 1º EM | 2º EM | 3º EM  ★ OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Turma (ex: A | B | C)  ★ OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Turno: Manhã | Tarde | Integral  ★ OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Data de nascimento no formato DD/MM/AAAA (ex: 15/03/2012)</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>E-mail do estudante (ex: ana.santos@portalsesisp.org.br)</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Número do RG do estudante (ex: 12.345.678-9)</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>UF emissora do RG (sigla, ex: SP)</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Órgão emissor do RG (ex: SSP)</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>CPF do estudante (ex: 123.456.789-00)</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>Status: Ativo (padrão) | Inativo | Transferido | Formado</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>Data de ingresso no formato DD/MM/AAAA (ex: 01/02/2024)</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Nome completo da mãe/responsável 1</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>Telefone da mãe/responsável 1 (ex: (16) 99999-8888)</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>E-mail da mãe/responsável 1</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>Nome completo do pai/responsável 2</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>Telefone do pai/responsável 2 (ex: (16) 98888-7777)</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>E-mail do pai/responsável 2</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>Nome completo da mãe / responsável 1</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>Telefone da mãe / responsável 1 (ex: (16) 99999-8888)</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>E-mail da mãe / responsável 1</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>Nome completo do pai / responsável 2</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>Telefone do pai / responsável 2 (ex: (16) 98888-7777)</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>E-mail do pai / responsável 2</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
         <is>
           <t>Endereço completo (ex: Rua das Flores, 123 — SJRP)</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="W2" s="6" t="inlineStr">
         <is>
           <t>Autorização LGPD: Sim | Não</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="X2" s="6" t="inlineStr">
         <is>
           <t>Foto já coletada: Sim | Não</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="Y2" s="6" t="inlineStr">
         <is>
           <t>Observações gerais sobre o estudante</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>006810</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>000120628062-1</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>ANA BEATRIZ SILVA SANTOS</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>6º Ano</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Manhã</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>15/03/2012</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>ana.santos@portalsesisp.org.br</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>12.345.678-9</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>SSP</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>123.456.789-00</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>01/02/2024</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>MARIA DA SILVA SANTOS</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="Q3" s="7" t="inlineStr">
         <is>
           <t>(16) 99999-8888</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="R3" s="7" t="inlineStr">
         <is>
           <t>maria.santos@email.com</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="S3" s="7" t="inlineStr">
         <is>
           <t>JOSÉ CARLOS SANTOS</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="T3" s="7" t="inlineStr">
         <is>
           <t>(16) 98888-7777</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="U3" s="7" t="inlineStr">
         <is>
           <t>jose.santos@email.com</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="V3" s="7" t="inlineStr">
         <is>
           <t>Rua das Flores, 123</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="W3" s="7" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="X3" s="7" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="Y3" s="7" t="inlineStr">
         <is>
           <t>Estudante com restrição alimentar</t>
         </is>
@@ -869,137 +1024,227 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="75" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>CARÔMETRO ESCOLAR — SESI 407</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Template de Importação de Estudantes</t>
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Template de Importação de Estudantes  |  v5.3</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="inlineStr"/>
+      <c r="A3" s="10" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>REGRAS GERAIS:</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>• Preencha a partir da linha 4 da aba 'Estudantes' (linhas 1-3 são cabeçalho+exemplo)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>• NÃO altere os nomes das colunas na linha 1</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>• Campos obrigatórios: rm_estudante, nome_estudante, serie, turma, turno</t>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>• Campos obrigatórios (★): rm_estudante, nome_estudante, serie, turma, turno</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="8" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>NOVOS CAMPOS  (v5.3):</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>• nu_chamada     → Número de chamada na turma (ex: 01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>• rg_estudante   → RG do estudante (ex: 12.345.678-9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>• uf_rg          → UF do RG (ex: SP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>• org_emissor_rg → Órgão emissor do RG (ex: SSP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>• cpf_estudante  → CPF do estudante (ex: 123.456.789-00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>FORMATOS:</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>• Datas: DD/MM/AAAA  (ex: 15/03/2012)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>• termo_autorizado / foto_coletada: Sim ou Não</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>• CPF: com ou sem formatação (o script formata automaticamente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>• serie: 6º Ano | 7º Ano | 8º Ano | 9º Ano | 1º EM | 2º EM | 3º EM</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>• turno: Manhã | Tarde | Integral</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>• status: Ativo | Inativo | Transferido | Formado</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>FOTOS:</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>• As fotos devem ser nomeadas como:  &lt;rm_estudante&gt;.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>• Exemplo: 006810.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>• Fotos nomeadas como: &lt;rm_estudante&gt;.jpg  (ex: 006810.jpg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>• Coloque todas as fotos na pasta  images/  do projeto</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>• O script organiza automaticamente as fotos por turma após a importação</t>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>• O script organiza automaticamente por turma após a importação</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>CORES DAS COLUNAS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>• Vermelho  → Identificação Escolar  (RM, RA, Nº Chamada, Nome, Série, Turma, Turno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>• Azul      → Dados Pessoais         (Nascimento, E-mail, RG, UF, Órgão, CPF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>• Verde     → Situação Escolar        (Status, Data Ingresso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>• Roxo      → Responsáveis           (Mãe/Pai — Nome, Telefone, E-mail)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>• Amarelo   → Endereço / Sistema      (Endereço, LGPD, Foto, Observações)</t>
         </is>
       </c>
     </row>

</xml_diff>